<commit_message>
Actualizacion datos REM VIH  1608
</commit_message>
<xml_diff>
--- a/2025/salida/P11_2025.xlsx
+++ b/2025/salida/P11_2025.xlsx
@@ -3466,7 +3466,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital San Juan de Dios (Santiago)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital San Juan de Dios (Santiago)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital San Juan de Dios (Santiago)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital San Juan de Dios (Santiago)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital San Juan de Dios (Santiago)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital San Juan de Dios (Santiago)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -8412,7 +8412,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -9144,7 +9144,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -9388,7 +9388,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -9692,7 +9692,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -9870,7 +9870,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -10388,7 +10388,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -10510,7 +10510,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -11451,7 +11451,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital San Juan de Dios (Santiago)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -11881,7 +11881,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur - Oriente</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>